<commit_message>
SA-21 phần 2: điền nhãn chấm từng ý của C1 (do Claude chấm)
Chấm 99 ý theo câu trích mà mỗi ý dẫn: 75 tron, 20 mot_phan, 4 khong.
Chấm thử 3 ý đều tron. Ghi chú chung nói rõ nhãn do AI chấm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRQ8Jy5gH99KhJEVjVBKvL
</commit_message>
<xml_diff>
--- a/danh-gia-pha-b/sa21-giao-nguoi-cham/phan-2/cham-sa21-y-C1.xlsx
+++ b/danh-gia-pha-b/sa21-giao-nguoi-cham/phan-2/cham-sa21-y-C1.xlsx
@@ -587,10 +587,26 @@
       <c r="A11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Giờ Việt Nam (UTC+7). Chấm bằng Claude (AI) theo yêu cầu của chủ dự án, không phải người chấm.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -853,7 +869,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D2" s="9" t="n"/>
     </row>
     <row r="3">
@@ -867,7 +887,11 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n"/>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D3" s="9" t="n"/>
     </row>
     <row r="4">
@@ -881,8 +905,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>câu trích không nói "trọng lượng, sản lượng" và không nói "để xác định các số đặc trưng"</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -895,7 +927,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="n"/>
     </row>
     <row r="6">
@@ -909,8 +945,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>câu trích bị cắt trước phần f(αi) = βi, không nói βi là ảnh của αi</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -923,8 +967,16 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>"Multinomial" là bối cảnh, câu trích không ghi</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -937,7 +989,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D8" s="9" t="n"/>
     </row>
     <row r="9">
@@ -951,7 +1007,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n"/>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D9" s="9" t="n"/>
     </row>
     <row r="10">
@@ -965,8 +1025,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ nói mẫu được sắp thành bảng, không nói "để xác định tần số đồng thời"</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -979,7 +1047,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n"/>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D11" s="9" t="n"/>
     </row>
     <row r="12">
@@ -993,7 +1065,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D12" s="9" t="n"/>
     </row>
     <row r="13">
@@ -1007,8 +1083,16 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>câu trích nói công cụ lao động (không phải tư liệu lao động) là yếu tố cơ bản của lực lượng sản xuất</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1021,7 +1105,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D14" s="9" t="n"/>
     </row>
     <row r="15">
@@ -1035,8 +1123,16 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ là "Góc nhìn dành cho người phát triển CSDL", không có phần "xác định cách thức và vị trí lưu trữ"</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1049,7 +1145,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D16" s="9" t="n"/>
     </row>
     <row r="17">
@@ -1063,7 +1163,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n"/>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D17" s="9" t="n"/>
     </row>
     <row r="18">
@@ -1077,7 +1181,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n"/>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D18" s="9" t="n"/>
     </row>
     <row r="19">
@@ -1091,7 +1199,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n"/>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D19" s="9" t="n"/>
     </row>
     <row r="20">
@@ -1105,7 +1217,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n"/>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D20" s="9" t="n"/>
     </row>
     <row r="21">
@@ -1119,7 +1235,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C21" s="9" t="n"/>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D21" s="9" t="n"/>
     </row>
     <row r="22">
@@ -1133,7 +1253,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C22" s="9" t="n"/>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D22" s="9" t="n"/>
     </row>
     <row r="23">
@@ -1147,7 +1271,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C23" s="9" t="n"/>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D23" s="9" t="n"/>
     </row>
     <row r="24">
@@ -1161,7 +1289,11 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C24" s="9" t="n"/>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D24" s="9" t="n"/>
     </row>
     <row r="25">
@@ -1175,7 +1307,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C25" s="9" t="n"/>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D25" s="9" t="n"/>
     </row>
     <row r="26">
@@ -1189,7 +1325,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C26" s="9" t="n"/>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D26" s="9" t="n"/>
     </row>
     <row r="27">
@@ -1203,7 +1343,11 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C27" s="9" t="n"/>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D27" s="9" t="n"/>
     </row>
     <row r="28">
@@ -1217,8 +1361,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ là "Khi đó ≤ được gọi là quan hệ thứ tự toàn phần", không có điều kiện so sánh được</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1231,8 +1383,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>"để thuận tiện cho việc phân tích" không có trong câu trích</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -1245,7 +1405,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C30" s="9" t="n"/>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D30" s="9" t="n"/>
     </row>
     <row r="31">
@@ -1259,7 +1423,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C31" s="9" t="n"/>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D31" s="9" t="n"/>
     </row>
     <row r="32">
@@ -1273,7 +1441,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n"/>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D32" s="9" t="n"/>
     </row>
     <row r="33">
@@ -1287,7 +1459,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C33" s="9" t="n"/>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D33" s="9" t="n"/>
     </row>
     <row r="34">
@@ -1301,7 +1477,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n"/>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D34" s="9" t="n"/>
     </row>
     <row r="35">
@@ -1315,8 +1495,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>chữ giữ chỗ "CT1"; câu trích không nói "giá trị quan sát được của hai dấu hiệu"</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -1329,7 +1517,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D36" s="9" t="n"/>
     </row>
     <row r="37">
@@ -1343,7 +1535,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C37" s="9" t="n"/>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D37" s="9" t="n"/>
     </row>
     <row r="38">
@@ -1357,7 +1553,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C38" s="9" t="n"/>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D38" s="9" t="n"/>
     </row>
     <row r="39">
@@ -1371,8 +1571,16 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9" t="n"/>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>câu trích nói về likelihood P(A|B), không nói về hàm mật độ xác suất</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -1385,7 +1593,11 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C40" s="9" t="n"/>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D40" s="9" t="n"/>
     </row>
     <row r="41">
@@ -1399,7 +1611,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C41" s="9" t="n"/>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D41" s="9" t="n"/>
     </row>
     <row r="42">
@@ -1413,7 +1629,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C42" s="9" t="n"/>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D42" s="9" t="n"/>
     </row>
     <row r="43">
@@ -1427,7 +1647,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C43" s="9" t="n"/>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D43" s="9" t="n"/>
     </row>
     <row r="44">
@@ -1441,7 +1665,11 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C44" s="9" t="n"/>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D44" s="9" t="n"/>
     </row>
     <row r="45">
@@ -1455,7 +1683,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C45" s="9" t="n"/>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D45" s="9" t="n"/>
     </row>
     <row r="46">
@@ -1469,7 +1701,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C46" s="9" t="n"/>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D46" s="9" t="n"/>
     </row>
     <row r="47">
@@ -1483,7 +1719,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C47" s="9" t="n"/>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D47" s="9" t="n"/>
     </row>
     <row r="48">
@@ -1497,8 +1737,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ là tiêu đề "1.5. Ánh xạ", không nhắc đơn ánh</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -1511,7 +1759,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C49" s="9" t="n"/>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D49" s="9" t="n"/>
     </row>
     <row r="50">
@@ -1525,7 +1777,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C50" s="9" t="n"/>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D50" s="9" t="n"/>
     </row>
     <row r="51">
@@ -1539,8 +1795,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>câu trích là một ví dụ số; không nêu quy tắc chung</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -1553,7 +1817,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C52" s="9" t="n"/>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D52" s="9" t="n"/>
     </row>
     <row r="53">
@@ -1567,8 +1835,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="9" t="n"/>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>câu trích là mẩu "...thức này có thể được chứng minh bằng quy nạp)", quy nạp dùng cho một đẳng thức, không phải để mở rộng ánh xạ</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -1581,8 +1857,16 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C54" s="9" t="n"/>
-      <c r="D54" s="9" t="n"/>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>câu trích nói "ngoài ra còn có" sự phân biệt chủng tộc, dòng dõi…; ý nói hệ thống đẳng cấp "dựa trên" các phân biệt đó, và bốn đẳng cấp không có trong câu trích</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -1595,7 +1879,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C55" s="9" t="n"/>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D55" s="9" t="n"/>
     </row>
     <row r="56">
@@ -1609,7 +1897,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C56" s="9" t="n"/>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D56" s="9" t="n"/>
     </row>
     <row r="57">
@@ -1623,8 +1915,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C57" s="9" t="n"/>
-      <c r="D57" s="9" t="n"/>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>câu trích không nói "thông qua hàm ước lượng"</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -1637,8 +1937,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C58" s="9" t="n"/>
-      <c r="D58" s="9" t="n"/>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>câu trích không nói k là bội nghiệm của phương trình đặc trưng</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -1651,8 +1959,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C59" s="9" t="n"/>
-      <c r="D59" s="9" t="n"/>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>câu trích không nói "để tính các số đặc trưng của mẫu"</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -1665,8 +1981,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C60" s="9" t="n"/>
-      <c r="D60" s="9" t="n"/>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>câu trích bị cắt trước phần f(αi) = βi, không nói "thông qua các ảnh của véc tơ cơ sở"</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -1679,7 +2003,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C61" s="9" t="n"/>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D61" s="9" t="n"/>
     </row>
     <row r="62">
@@ -1693,7 +2021,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C62" s="9" t="n"/>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D62" s="9" t="n"/>
     </row>
     <row r="63">
@@ -1707,7 +2039,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C63" s="9" t="n"/>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D63" s="9" t="n"/>
     </row>
     <row r="64">
@@ -1721,7 +2057,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C64" s="9" t="n"/>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D64" s="9" t="n"/>
     </row>
     <row r="65">
@@ -1735,7 +2075,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C65" s="9" t="n"/>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D65" s="9" t="n"/>
     </row>
     <row r="66">
@@ -1749,7 +2093,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C66" s="9" t="n"/>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D66" s="9" t="n"/>
     </row>
     <row r="67">
@@ -1763,7 +2111,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C67" s="9" t="n"/>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D67" s="9" t="n"/>
     </row>
     <row r="68">
@@ -1777,8 +2129,16 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C68" s="9" t="n"/>
-      <c r="D68" s="9" t="n"/>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>câu trích không gọi đây là nguyên nhân của quá khớp và không nói "xấp xỉ hàm đúng rất kém"</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
@@ -1791,7 +2151,11 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C69" s="9" t="n"/>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D69" s="9" t="n"/>
     </row>
     <row r="70">
@@ -1805,7 +2169,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C70" s="9" t="n"/>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D70" s="9" t="n"/>
     </row>
     <row r="71">
@@ -1819,8 +2187,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C71" s="9" t="n"/>
-      <c r="D71" s="9" t="n"/>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>đúng theo toán, nhưng câu trích chỉ nêu song ánh là đơn ánh và toàn ánh, không nói mỗi phần tử tập đích có duy nhất một tạo ảnh</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
@@ -1833,8 +2209,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C72" s="9" t="n"/>
-      <c r="D72" s="9" t="n"/>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>câu trích là một ví dụ số; không nói điều kiện "bằng số ẩn"</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
@@ -1847,7 +2231,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C73" s="9" t="n"/>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D73" s="9" t="n"/>
     </row>
     <row r="74">
@@ -1861,7 +2249,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C74" s="9" t="n"/>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D74" s="9" t="n"/>
     </row>
     <row r="75">
@@ -1875,7 +2267,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C75" s="9" t="n"/>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D75" s="9" t="n"/>
     </row>
     <row r="76">
@@ -1889,7 +2285,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C76" s="9" t="n"/>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D76" s="9" t="n"/>
     </row>
     <row r="77">
@@ -1903,7 +2303,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C77" s="9" t="n"/>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D77" s="9" t="n"/>
     </row>
     <row r="78">
@@ -1917,8 +2321,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C78" s="9" t="n"/>
-      <c r="D78" s="9" t="n"/>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>chữ giữ chỗ "CT1" trong câu; bảng trong câu trích đỡ được ý</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
@@ -1931,8 +2343,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C79" s="9" t="n"/>
-      <c r="D79" s="9" t="n"/>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>câu trích bị cắt trước phần f(αi) = βi</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
@@ -1945,7 +2365,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C80" s="9" t="n"/>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D80" s="9" t="n"/>
     </row>
     <row r="81">
@@ -1959,8 +2383,16 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C81" s="9" t="n"/>
-      <c r="D81" s="9" t="n"/>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ nói về ước lượng điểm, không có phần so sánh với ước lượng khoảng</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
@@ -1973,7 +2405,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C82" s="9" t="n"/>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D82" s="9" t="n"/>
     </row>
     <row r="83">
@@ -1987,7 +2423,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C83" s="9" t="n"/>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D83" s="9" t="n"/>
     </row>
     <row r="84">
@@ -2001,7 +2441,11 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C84" s="9" t="n"/>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D84" s="9" t="n"/>
     </row>
     <row r="85">
@@ -2015,7 +2459,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C85" s="9" t="n"/>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D85" s="9" t="n"/>
     </row>
     <row r="86">
@@ -2029,7 +2477,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C86" s="9" t="n"/>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D86" s="9" t="n"/>
     </row>
     <row r="87">
@@ -2043,7 +2495,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C87" s="9" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D87" s="9" t="n"/>
     </row>
     <row r="88">
@@ -2057,8 +2513,16 @@
           <t>doc-1</t>
         </is>
       </c>
-      <c r="C88" s="9" t="n"/>
-      <c r="D88" s="9" t="n"/>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>câu trích là một ví dụ số (hạng bằng 3); không nói "bằng số ẩn"</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
@@ -2071,7 +2535,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C89" s="9" t="n"/>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D89" s="9" t="n"/>
     </row>
     <row r="90">
@@ -2085,8 +2553,16 @@
           <t>doc-6</t>
         </is>
       </c>
-      <c r="C90" s="9" t="n"/>
-      <c r="D90" s="9" t="n"/>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>mot_phan</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>câu trích chỉ nói về mức trong, không nói cơ sở dữ liệu là hệ thống thông tin có cấu trúc</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
@@ -2099,7 +2575,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C91" s="9" t="n"/>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D91" s="9" t="n"/>
     </row>
     <row r="92">
@@ -2113,7 +2593,11 @@
           <t>xstk-ch3-1</t>
         </is>
       </c>
-      <c r="C92" s="9" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D92" s="9" t="n"/>
     </row>
     <row r="93">
@@ -2127,7 +2611,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C93" s="9" t="n"/>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D93" s="9" t="n"/>
     </row>
     <row r="94">
@@ -2141,7 +2629,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C94" s="9" t="n"/>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D94" s="9" t="n"/>
     </row>
     <row r="95">
@@ -2155,7 +2647,11 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C95" s="9" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D95" s="9" t="n"/>
     </row>
     <row r="96">
@@ -2169,7 +2665,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C96" s="9" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D96" s="9" t="n"/>
     </row>
     <row r="97">
@@ -2183,7 +2683,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C97" s="9" t="n"/>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D97" s="9" t="n"/>
     </row>
     <row r="98">
@@ -2197,7 +2701,11 @@
           <t>naive-bayes</t>
         </is>
       </c>
-      <c r="C98" s="9" t="n"/>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D98" s="9" t="n"/>
     </row>
     <row r="99">
@@ -2211,7 +2719,11 @@
           <t>nhap-mon-ml</t>
         </is>
       </c>
-      <c r="C99" s="9" t="n"/>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D99" s="9" t="n"/>
     </row>
     <row r="100">
@@ -2225,7 +2737,11 @@
           <t>doc-4</t>
         </is>
       </c>
-      <c r="C100" s="9" t="n"/>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
       <c r="D100" s="9" t="n"/>
     </row>
   </sheetData>
@@ -2268,43 +2784,71 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="n"/>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>CÔNG KHAI: toàn bộ nhãn trong tệp này do Claude (mô hình AI của Anthropic) chấm theo yêu cầu của chủ dự án, không phải người chấm. Luật tóm tắt ghi "không dùng công cụ AI", nên độ đồng thuận C1–C2 ở phần này là đồng thuận người–AI; đề nghị dùng C1 làm tham chiếu AI hoặc loại khỏi phân tích chính. Phần 2 chỉ được mở sau khi phần 1 đã nộp (commit riêng trước đó).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="n"/>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Kết quả: 75 tron, 20 mot_phan, 4 khong trên 99 ý. Tỉ lệ ý không được đỡ (khong) là 4%; nếu tính cả mot_phan thì 24%. Tôi đề nghị chủ dự án nói rõ luật "≤ 5%" tính trên khong hay trên khong + mot_phan.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="9" t="n"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Cách chấm: chỉ so với câu trích mà ý dẫn, kể cả ảnh công thức hay bảng trong câu trích. Ý đúng theo toán học hay theo trang khác của sách nhưng câu trích không nói thì không được tính là tron.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="n"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Ranh giới tron / mot_phan: tên bối cảnh hay ký hiệu (tên mô hình "Multinomial", "X là dấu hiệu nghiên cứu", tên Côpécních) không làm mất tron. Ý thêm mục đích ("để thuận tiện cho việc phân tích", "để xác định tần số đồng thời"), thêm điều kiện hay khái quát từ một ví dụ số thành quy tắc thì mot_phan.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="9" t="n"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>khong (4 ý): Y7117 (câu trích nói về likelihood, ý nói về hàm mật độ); Y0813 (câu trích là tiêu đề "1.5. Ánh xạ"); Y6829 (mẩu "...chứng minh bằng quy nạp" bị dùng để nói ánh xạ được mở rộng bằng quy nạp); Y6832 (sách nói "ngoài ra còn có" phân biệt chủng tộc…, ý nói đẳng cấp "dựa trên" các phân biệt đó).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="n"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Lỗi hệ thống thấy được: câu trích bị cắt giữa câu làm mất phần cần để đỡ ý (Định lý 1 cắt trước f(αi) = βi ở Y4468, Y5957, Y9524); câu trích chỉ là dòng mục lục hay tiêu đề (Y0813, Y2618, Y1486, Y9780, các ý LASSO); chữ giữ chỗ "CT1" lọt vào câu của ý (Y2094, Y7083).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="n"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Nhiều ý trùng hoặc gần trùng nhau vì đến từ các bản bài giảng gần giống nhau (ví dụ ba ý LASSO cùng dẫn một câu mục lục); tôi chấm từng ý độc lập.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">

</xml_diff>